<commit_message>
Update 00981A report 2026-06-22
</commit_message>
<xml_diff>
--- a/etf_data/49YTW_20260622.xlsx
+++ b/etf_data/49YTW_20260622.xlsx
@@ -12,9 +12,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="213">
-  <si>
-    <t xml:space="preserve">資料日期：115/06/18</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="208">
+  <si>
+    <t xml:space="preserve">資料日期：115/06/22</t>
   </si>
   <si>
     <t xml:space="preserve">基金資產</t>
@@ -23,19 +23,19 @@
     <t xml:space="preserve">淨資產</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 297,710,073,788</t>
+    <t xml:space="preserve">NTD 300,179,846,772</t>
   </si>
   <si>
     <t xml:space="preserve">流通在外單位數</t>
   </si>
   <si>
-    <t xml:space="preserve">9,412,709,000</t>
+    <t xml:space="preserve">9,299,709,000</t>
   </si>
   <si>
     <t xml:space="preserve">每單位淨值</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 31.63</t>
+    <t xml:space="preserve">NTD 32.28</t>
   </si>
   <si>
     <t xml:space="preserve">項目</t>
@@ -59,34 +59,34 @@
     <t xml:space="preserve">股票</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 296,698,261,500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">99.66%</t>
+    <t xml:space="preserve">NTD 297,131,794,420</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98.98%</t>
   </si>
   <si>
     <t xml:space="preserve">現金</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 4,491,865,572</t>
+    <t xml:space="preserve">NTD 4,661,064,427</t>
   </si>
   <si>
     <t xml:space="preserve">期貨保證金</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 500,128,241</t>
+    <t xml:space="preserve">NTD 500,781,127</t>
   </si>
   <si>
     <t xml:space="preserve">附買回債券</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 5,085,473,246</t>
+    <t xml:space="preserve">NTD 4,038,000,000</t>
   </si>
   <si>
     <t xml:space="preserve">應收付證券款</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD -3,023,511,393</t>
+    <t xml:space="preserve">NTD 3,114,260,153</t>
   </si>
   <si>
     <t xml:space="preserve">股票代號</t>
@@ -110,7 +110,19 @@
     <t xml:space="preserve">11,960,000</t>
   </si>
   <si>
-    <t xml:space="preserve">9.68%</t>
+    <t xml:space="preserve">10.00%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2383</t>
+  </si>
+  <si>
+    <t xml:space="preserve">台光電</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,486,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.71%</t>
   </si>
   <si>
     <t xml:space="preserve">2327</t>
@@ -122,19 +134,7 @@
     <t xml:space="preserve">23,892,000</t>
   </si>
   <si>
-    <t xml:space="preserve">8.67%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2383</t>
-  </si>
-  <si>
-    <t xml:space="preserve">台光電</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,486,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.44%</t>
+    <t xml:space="preserve">8.48%</t>
   </si>
   <si>
     <t xml:space="preserve">2454</t>
@@ -146,7 +146,7 @@
     <t xml:space="preserve">4,861,000</t>
   </si>
   <si>
-    <t xml:space="preserve">7.17%</t>
+    <t xml:space="preserve">7.23%</t>
   </si>
   <si>
     <t xml:space="preserve">2345</t>
@@ -158,7 +158,7 @@
     <t xml:space="preserve">6,334,000</t>
   </si>
   <si>
-    <t xml:space="preserve">5.18%</t>
+    <t xml:space="preserve">5.48%</t>
   </si>
   <si>
     <t xml:space="preserve">6223</t>
@@ -170,7 +170,7 @@
     <t xml:space="preserve">2,279,000</t>
   </si>
   <si>
-    <t xml:space="preserve">4.91%</t>
+    <t xml:space="preserve">4.88%</t>
   </si>
   <si>
     <t xml:space="preserve">2308</t>
@@ -179,10 +179,43 @@
     <t xml:space="preserve">台達電</t>
   </si>
   <si>
-    <t xml:space="preserve">6,572,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.75%</t>
+    <t xml:space="preserve">6,222,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.46%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">欣興</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13,307,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">奇鋐</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,191,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.18%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2303</t>
+  </si>
+  <si>
+    <t xml:space="preserve">聯電</t>
+  </si>
+  <si>
+    <t xml:space="preserve">77,390,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.12%</t>
   </si>
   <si>
     <t xml:space="preserve">6669</t>
@@ -194,31 +227,16 @@
     <t xml:space="preserve">2,492,000</t>
   </si>
   <si>
-    <t xml:space="preserve">4.29%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">奇鋐</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,191,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.18%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3037</t>
-  </si>
-  <si>
-    <t xml:space="preserve">欣興</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12,466,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.05%</t>
+    <t xml:space="preserve">4.03%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3711</t>
+  </si>
+  <si>
+    <t xml:space="preserve">日月光投控</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17,948,000</t>
   </si>
   <si>
     <t xml:space="preserve">2368</t>
@@ -230,28 +248,7 @@
     <t xml:space="preserve">8,315,000</t>
   </si>
   <si>
-    <t xml:space="preserve">3.78%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2303</t>
-  </si>
-  <si>
-    <t xml:space="preserve">聯電</t>
-  </si>
-  <si>
-    <t xml:space="preserve">77,390,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3711</t>
-  </si>
-  <si>
-    <t xml:space="preserve">日月光投控</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17,948,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.70%</t>
+    <t xml:space="preserve">3.86%</t>
   </si>
   <si>
     <t xml:space="preserve">3665</t>
@@ -263,7 +260,40 @@
     <t xml:space="preserve">4,833,848</t>
   </si>
   <si>
-    <t xml:space="preserve">3.41%</t>
+    <t xml:space="preserve">3.20%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6274</t>
+  </si>
+  <si>
+    <t xml:space="preserve">台燿</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,058,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3653</t>
+  </si>
+  <si>
+    <t xml:space="preserve">健策</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,267,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.90%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5274</t>
+  </si>
+  <si>
+    <t xml:space="preserve">信驊</t>
+  </si>
+  <si>
+    <t xml:space="preserve">422,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.71%</t>
   </si>
   <si>
     <t xml:space="preserve">8046</t>
@@ -272,46 +302,22 @@
     <t xml:space="preserve">南電</t>
   </si>
   <si>
-    <t xml:space="preserve">10,828,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.18%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6274</t>
-  </si>
-  <si>
-    <t xml:space="preserve">台燿</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,058,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.12%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3653</t>
-  </si>
-  <si>
-    <t xml:space="preserve">健策</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,267,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.02%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5274</t>
-  </si>
-  <si>
-    <t xml:space="preserve">信驊</t>
-  </si>
-  <si>
-    <t xml:space="preserve">422,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.69%</t>
+    <t xml:space="preserve">8,917,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.57%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">富世達</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,811,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.10%</t>
   </si>
   <si>
     <t xml:space="preserve">6515</t>
@@ -320,10 +326,7 @@
     <t xml:space="preserve">穎崴</t>
   </si>
   <si>
-    <t xml:space="preserve">436,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.38%</t>
+    <t xml:space="preserve">348,000</t>
   </si>
   <si>
     <t xml:space="preserve">6510</t>
@@ -335,19 +338,7 @@
     <t xml:space="preserve">930,000</t>
   </si>
   <si>
-    <t xml:space="preserve">1.13%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">富世達</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,811,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.07%</t>
+    <t xml:space="preserve">1.09%</t>
   </si>
   <si>
     <t xml:space="preserve">8210</t>
@@ -356,7 +347,7 @@
     <t xml:space="preserve">勤誠</t>
   </si>
   <si>
-    <t xml:space="preserve">1.04%</t>
+    <t xml:space="preserve">1.03%</t>
   </si>
   <si>
     <t xml:space="preserve">2449</t>
@@ -368,7 +359,7 @@
     <t xml:space="preserve">6,484,000</t>
   </si>
   <si>
-    <t xml:space="preserve">0.67%</t>
+    <t xml:space="preserve">0.73%</t>
   </si>
   <si>
     <t xml:space="preserve">3533</t>
@@ -392,37 +383,205 @@
     <t xml:space="preserve">7,307,000</t>
   </si>
   <si>
+    <t xml:space="preserve">0.65%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6147</t>
+  </si>
+  <si>
+    <t xml:space="preserve">頎邦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,275,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.58%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6187</t>
+  </si>
+  <si>
+    <t xml:space="preserve">萬潤</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,334,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.56%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8150</t>
+  </si>
+  <si>
+    <t xml:space="preserve">南茂</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11,635,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.44%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5439</t>
+  </si>
+  <si>
+    <t xml:space="preserve">高技</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,528,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.39%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4966</t>
+  </si>
+  <si>
+    <t xml:space="preserve">譜瑞-KY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,642,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.38%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6278</t>
+  </si>
+  <si>
+    <t xml:space="preserve">台表科</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,334,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6271</t>
+  </si>
+  <si>
+    <t xml:space="preserve">同欣電</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,966,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.26%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1590</t>
+  </si>
+  <si>
+    <t xml:space="preserve">亞德客-KY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">530,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.25%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8358</t>
+  </si>
+  <si>
+    <t xml:space="preserve">金居</t>
+  </si>
+  <si>
+    <t xml:space="preserve">980,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.23%</t>
+  </si>
+  <si>
     <t xml:space="preserve">8996</t>
   </si>
   <si>
     <t xml:space="preserve">高力</t>
   </si>
   <si>
-    <t xml:space="preserve">1,034,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.55%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6187</t>
-  </si>
-  <si>
-    <t xml:space="preserve">萬潤</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,334,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6147</t>
-  </si>
-  <si>
-    <t xml:space="preserve">頎邦</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6,275,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.53%</t>
+    <t xml:space="preserve">354,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.18%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6191</t>
+  </si>
+  <si>
+    <t xml:space="preserve">精成科</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,988,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.14%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6488</t>
+  </si>
+  <si>
+    <t xml:space="preserve">環球晶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">350,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.13%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3264</t>
+  </si>
+  <si>
+    <t xml:space="preserve">欣銓</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,508,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.12%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3376</t>
+  </si>
+  <si>
+    <t xml:space="preserve">新日興</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,741,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">中鋼</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,163,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.03%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3661</t>
+  </si>
+  <si>
+    <t xml:space="preserve">世芯-KY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.00%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1815</t>
+  </si>
+  <si>
+    <t xml:space="preserve">富喬</t>
+  </si>
+  <si>
+    <t xml:space="preserve">107,000</t>
   </si>
   <si>
     <t xml:space="preserve">3443</t>
@@ -431,46 +590,19 @@
     <t xml:space="preserve">創意</t>
   </si>
   <si>
-    <t xml:space="preserve">258,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.42%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8150</t>
-  </si>
-  <si>
-    <t xml:space="preserve">南茂</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11,635,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.41%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5439</t>
-  </si>
-  <si>
-    <t xml:space="preserve">高技</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,528,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.39%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4966</t>
-  </si>
-  <si>
-    <t xml:space="preserve">譜瑞-KY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,642,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.38%</t>
+    <t xml:space="preserve">2439</t>
+  </si>
+  <si>
+    <t xml:space="preserve">美律</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">大立光</t>
   </si>
   <si>
     <t xml:space="preserve">4958</t>
@@ -479,163 +611,16 @@
     <t xml:space="preserve">臻鼎-KY</t>
   </si>
   <si>
-    <t xml:space="preserve">1,428,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.31%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6278</t>
-  </si>
-  <si>
-    <t xml:space="preserve">台表科</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,334,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.30%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1590</t>
-  </si>
-  <si>
-    <t xml:space="preserve">亞德客-KY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">530,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.25%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8358</t>
-  </si>
-  <si>
-    <t xml:space="preserve">金居</t>
-  </si>
-  <si>
-    <t xml:space="preserve">980,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.23%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6271</t>
-  </si>
-  <si>
-    <t xml:space="preserve">同欣電</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,966,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.16%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6191</t>
-  </si>
-  <si>
-    <t xml:space="preserve">精成科</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,988,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.13%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6488</t>
-  </si>
-  <si>
-    <t xml:space="preserve">環球晶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">350,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3264</t>
-  </si>
-  <si>
-    <t xml:space="preserve">欣銓</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,508,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.12%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3376</t>
-  </si>
-  <si>
-    <t xml:space="preserve">新日興</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,741,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">中鋼</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,163,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.03%</t>
+    <t xml:space="preserve">2382</t>
+  </si>
+  <si>
+    <t xml:space="preserve">廣達</t>
   </si>
   <si>
     <t xml:space="preserve">2313</t>
   </si>
   <si>
     <t xml:space="preserve">華通</t>
-  </si>
-  <si>
-    <t xml:space="preserve">329,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3661</t>
-  </si>
-  <si>
-    <t xml:space="preserve">世芯-KY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.00%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1815</t>
-  </si>
-  <si>
-    <t xml:space="preserve">富喬</t>
-  </si>
-  <si>
-    <t xml:space="preserve">107,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2439</t>
-  </si>
-  <si>
-    <t xml:space="preserve">美律</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">大立光</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2382</t>
-  </si>
-  <si>
-    <t xml:space="preserve">廣達</t>
   </si>
   <si>
     <t xml:space="preserve">5347</t>
@@ -1430,7 +1415,7 @@
   <dimension ref="A1:E70"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.9" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="1" max="1" width="24.75" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="2" max="2" width="24.75" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="3" max="3" width="12.9" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="4" max="4" width="10.35" bestFit="1" customWidth="1" collapsed="1"/>
@@ -1684,469 +1669,469 @@
         <v>59</v>
       </c>
       <c r="D28" s="62" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="63" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" s="64" t="s">
         <v>61</v>
       </c>
-      <c r="B29" s="64" t="s">
+      <c r="C29" s="65" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="65" t="s">
+      <c r="D29" s="66" t="s">
         <v>63</v>
-      </c>
-      <c r="D29" s="66" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="67" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="68" t="s">
         <v>65</v>
       </c>
-      <c r="B30" s="68" t="s">
+      <c r="C30" s="69" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="69" t="s">
+      <c r="D30" s="70" t="s">
         <v>67</v>
-      </c>
-      <c r="D30" s="70" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="71" t="s">
+        <v>68</v>
+      </c>
+      <c r="B31" s="72" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="72" t="s">
+      <c r="C31" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="C31" s="73" t="s">
+      <c r="D31" s="74" t="s">
         <v>71</v>
-      </c>
-      <c r="D31" s="74" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="75" t="s">
+        <v>72</v>
+      </c>
+      <c r="B32" s="76" t="s">
         <v>73</v>
       </c>
-      <c r="B32" s="76" t="s">
+      <c r="C32" s="77" t="s">
         <v>74</v>
       </c>
-      <c r="C32" s="77" t="s">
-        <v>75</v>
-      </c>
       <c r="D32" s="78" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="79" t="s">
+        <v>75</v>
+      </c>
+      <c r="B33" s="80" t="s">
         <v>76</v>
       </c>
-      <c r="B33" s="80" t="s">
+      <c r="C33" s="81" t="s">
         <v>77</v>
       </c>
-      <c r="C33" s="81" t="s">
+      <c r="D33" s="82" t="s">
         <v>78</v>
-      </c>
-      <c r="D33" s="82" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="83" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" s="84" t="s">
         <v>80</v>
       </c>
-      <c r="B34" s="84" t="s">
+      <c r="C34" s="85" t="s">
         <v>81</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="D34" s="86" t="s">
         <v>82</v>
-      </c>
-      <c r="D34" s="86" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="87" t="s">
+        <v>83</v>
+      </c>
+      <c r="B35" s="88" t="s">
         <v>84</v>
       </c>
-      <c r="B35" s="88" t="s">
+      <c r="C35" s="89" t="s">
         <v>85</v>
       </c>
-      <c r="C35" s="89" t="s">
-        <v>86</v>
-      </c>
       <c r="D35" s="90" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="91" t="s">
+        <v>86</v>
+      </c>
+      <c r="B36" s="92" t="s">
+        <v>87</v>
+      </c>
+      <c r="C36" s="93" t="s">
         <v>88</v>
       </c>
-      <c r="B36" s="92" t="s">
+      <c r="D36" s="94" t="s">
         <v>89</v>
-      </c>
-      <c r="C36" s="93" t="s">
-        <v>90</v>
-      </c>
-      <c r="D36" s="94" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="95" t="s">
+        <v>90</v>
+      </c>
+      <c r="B37" s="96" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" s="97" t="s">
         <v>92</v>
       </c>
-      <c r="B37" s="96" t="s">
+      <c r="D37" s="98" t="s">
         <v>93</v>
-      </c>
-      <c r="C37" s="97" t="s">
-        <v>94</v>
-      </c>
-      <c r="D37" s="98" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="99" t="s">
+        <v>94</v>
+      </c>
+      <c r="B38" s="100" t="s">
+        <v>95</v>
+      </c>
+      <c r="C38" s="101" t="s">
         <v>96</v>
       </c>
-      <c r="B38" s="100" t="s">
+      <c r="D38" s="102" t="s">
         <v>97</v>
-      </c>
-      <c r="C38" s="101" t="s">
-        <v>98</v>
-      </c>
-      <c r="D38" s="102" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="103" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" s="104" t="s">
+        <v>99</v>
+      </c>
+      <c r="C39" s="105" t="s">
         <v>100</v>
       </c>
-      <c r="B39" s="104" t="s">
+      <c r="D39" s="106" t="s">
         <v>101</v>
-      </c>
-      <c r="C39" s="105" t="s">
-        <v>102</v>
-      </c>
-      <c r="D39" s="106" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="107" t="s">
+        <v>102</v>
+      </c>
+      <c r="B40" s="108" t="s">
+        <v>103</v>
+      </c>
+      <c r="C40" s="109" t="s">
         <v>104</v>
       </c>
-      <c r="B40" s="108" t="s">
-        <v>105</v>
-      </c>
-      <c r="C40" s="109" t="s">
-        <v>106</v>
-      </c>
       <c r="D40" s="110" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="111" t="s">
+        <v>105</v>
+      </c>
+      <c r="B41" s="112" t="s">
+        <v>106</v>
+      </c>
+      <c r="C41" s="113" t="s">
+        <v>107</v>
+      </c>
+      <c r="D41" s="114" t="s">
         <v>108</v>
-      </c>
-      <c r="B41" s="112" t="s">
-        <v>109</v>
-      </c>
-      <c r="C41" s="113" t="s">
-        <v>110</v>
-      </c>
-      <c r="D41" s="114" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="115" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B42" s="116" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C42" s="117" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="D42" s="118" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="119" t="s">
+        <v>112</v>
+      </c>
+      <c r="B43" s="120" t="s">
+        <v>113</v>
+      </c>
+      <c r="C43" s="121" t="s">
+        <v>114</v>
+      </c>
+      <c r="D43" s="122" t="s">
         <v>115</v>
-      </c>
-      <c r="B43" s="120" t="s">
-        <v>116</v>
-      </c>
-      <c r="C43" s="121" t="s">
-        <v>117</v>
-      </c>
-      <c r="D43" s="122" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="123" t="s">
+        <v>116</v>
+      </c>
+      <c r="B44" s="124" t="s">
+        <v>117</v>
+      </c>
+      <c r="C44" s="125" t="s">
+        <v>118</v>
+      </c>
+      <c r="D44" s="126" t="s">
         <v>119</v>
-      </c>
-      <c r="B44" s="124" t="s">
-        <v>120</v>
-      </c>
-      <c r="C44" s="125" t="s">
-        <v>121</v>
-      </c>
-      <c r="D44" s="126" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="127" t="s">
+        <v>120</v>
+      </c>
+      <c r="B45" s="128" t="s">
+        <v>121</v>
+      </c>
+      <c r="C45" s="129" t="s">
+        <v>122</v>
+      </c>
+      <c r="D45" s="130" t="s">
         <v>123</v>
-      </c>
-      <c r="B45" s="128" t="s">
-        <v>124</v>
-      </c>
-      <c r="C45" s="129" t="s">
-        <v>125</v>
-      </c>
-      <c r="D45" s="130" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="131" t="s">
+        <v>124</v>
+      </c>
+      <c r="B46" s="132" t="s">
+        <v>125</v>
+      </c>
+      <c r="C46" s="133" t="s">
         <v>126</v>
       </c>
-      <c r="B46" s="132" t="s">
+      <c r="D46" s="134" t="s">
         <v>127</v>
-      </c>
-      <c r="C46" s="133" t="s">
-        <v>128</v>
-      </c>
-      <c r="D46" s="134" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="135" t="s">
+        <v>128</v>
+      </c>
+      <c r="B47" s="136" t="s">
+        <v>129</v>
+      </c>
+      <c r="C47" s="137" t="s">
         <v>130</v>
       </c>
-      <c r="B47" s="136" t="s">
+      <c r="D47" s="138" t="s">
         <v>131</v>
-      </c>
-      <c r="C47" s="137" t="s">
-        <v>132</v>
-      </c>
-      <c r="D47" s="138" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="139" t="s">
+        <v>132</v>
+      </c>
+      <c r="B48" s="140" t="s">
         <v>133</v>
       </c>
-      <c r="B48" s="140" t="s">
+      <c r="C48" s="141" t="s">
         <v>134</v>
       </c>
-      <c r="C48" s="141" t="s">
+      <c r="D48" s="142" t="s">
         <v>135</v>
-      </c>
-      <c r="D48" s="142" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="143" t="s">
+        <v>136</v>
+      </c>
+      <c r="B49" s="144" t="s">
         <v>137</v>
       </c>
-      <c r="B49" s="144" t="s">
+      <c r="C49" s="145" t="s">
         <v>138</v>
       </c>
-      <c r="C49" s="145" t="s">
+      <c r="D49" s="146" t="s">
         <v>139</v>
-      </c>
-      <c r="D49" s="146" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="147" t="s">
+        <v>140</v>
+      </c>
+      <c r="B50" s="148" t="s">
         <v>141</v>
       </c>
-      <c r="B50" s="148" t="s">
+      <c r="C50" s="149" t="s">
         <v>142</v>
       </c>
-      <c r="C50" s="149" t="s">
+      <c r="D50" s="150" t="s">
         <v>143</v>
-      </c>
-      <c r="D50" s="150" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="151" t="s">
+        <v>144</v>
+      </c>
+      <c r="B51" s="152" t="s">
         <v>145</v>
       </c>
-      <c r="B51" s="152" t="s">
+      <c r="C51" s="153" t="s">
         <v>146</v>
       </c>
-      <c r="C51" s="153" t="s">
+      <c r="D51" s="154" t="s">
         <v>147</v>
-      </c>
-      <c r="D51" s="154" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="155" t="s">
+        <v>148</v>
+      </c>
+      <c r="B52" s="156" t="s">
         <v>149</v>
       </c>
-      <c r="B52" s="156" t="s">
+      <c r="C52" s="157" t="s">
         <v>150</v>
       </c>
-      <c r="C52" s="157" t="s">
+      <c r="D52" s="158" t="s">
         <v>151</v>
-      </c>
-      <c r="D52" s="158" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="159" t="s">
+        <v>152</v>
+      </c>
+      <c r="B53" s="160" t="s">
         <v>153</v>
       </c>
-      <c r="B53" s="160" t="s">
+      <c r="C53" s="161" t="s">
         <v>154</v>
       </c>
-      <c r="C53" s="161" t="s">
+      <c r="D53" s="162" t="s">
         <v>155</v>
-      </c>
-      <c r="D53" s="162" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="163" t="s">
+        <v>156</v>
+      </c>
+      <c r="B54" s="164" t="s">
         <v>157</v>
       </c>
-      <c r="B54" s="164" t="s">
+      <c r="C54" s="165" t="s">
         <v>158</v>
       </c>
-      <c r="C54" s="165" t="s">
+      <c r="D54" s="166" t="s">
         <v>159</v>
-      </c>
-      <c r="D54" s="166" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="167" t="s">
+        <v>160</v>
+      </c>
+      <c r="B55" s="168" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="168" t="s">
+      <c r="C55" s="169" t="s">
         <v>162</v>
       </c>
-      <c r="C55" s="169" t="s">
+      <c r="D55" s="170" t="s">
         <v>163</v>
-      </c>
-      <c r="D55" s="170" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="171" t="s">
+        <v>164</v>
+      </c>
+      <c r="B56" s="172" t="s">
         <v>165</v>
       </c>
-      <c r="B56" s="172" t="s">
+      <c r="C56" s="173" t="s">
         <v>166</v>
       </c>
-      <c r="C56" s="173" t="s">
+      <c r="D56" s="174" t="s">
         <v>167</v>
-      </c>
-      <c r="D56" s="174" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="175" t="s">
+        <v>168</v>
+      </c>
+      <c r="B57" s="176" t="s">
         <v>169</v>
       </c>
-      <c r="B57" s="176" t="s">
+      <c r="C57" s="177" t="s">
         <v>170</v>
       </c>
-      <c r="C57" s="177" t="s">
+      <c r="D57" s="178" t="s">
         <v>171</v>
-      </c>
-      <c r="D57" s="178" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="179" t="s">
+        <v>172</v>
+      </c>
+      <c r="B58" s="180" t="s">
         <v>173</v>
       </c>
-      <c r="B58" s="180" t="s">
+      <c r="C58" s="181" t="s">
         <v>174</v>
       </c>
-      <c r="C58" s="181" t="s">
+      <c r="D58" s="182" t="s">
         <v>175</v>
-      </c>
-      <c r="D58" s="182" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="183" t="s">
+        <v>176</v>
+      </c>
+      <c r="B59" s="184" t="s">
         <v>177</v>
       </c>
-      <c r="B59" s="184" t="s">
+      <c r="C59" s="185" t="s">
         <v>178</v>
       </c>
-      <c r="C59" s="185" t="s">
-        <v>179</v>
-      </c>
       <c r="D59" s="186" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="187" t="s">
+        <v>179</v>
+      </c>
+      <c r="B60" s="188" t="s">
         <v>180</v>
       </c>
-      <c r="B60" s="188" t="s">
+      <c r="C60" s="189" t="s">
         <v>181</v>
       </c>
-      <c r="C60" s="189" t="s">
+      <c r="D60" s="190" t="s">
         <v>182</v>
-      </c>
-      <c r="D60" s="190" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="191" t="s">
+        <v>183</v>
+      </c>
+      <c r="B61" s="192" t="s">
         <v>184</v>
       </c>
-      <c r="B61" s="192" t="s">
+      <c r="C61" s="193" t="s">
         <v>185</v>
       </c>
-      <c r="C61" s="193" t="s">
+      <c r="D61" s="194" t="s">
         <v>186</v>
-      </c>
-      <c r="D61" s="194" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="62">
@@ -2160,119 +2145,119 @@
         <v>189</v>
       </c>
       <c r="D62" s="198" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="199" t="s">
+        <v>190</v>
+      </c>
+      <c r="B63" s="200" t="s">
         <v>191</v>
       </c>
-      <c r="B63" s="200" t="s">
-        <v>192</v>
-      </c>
       <c r="C63" s="201" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="D63" s="202" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="203" t="s">
+        <v>192</v>
+      </c>
+      <c r="B64" s="204" t="s">
+        <v>193</v>
+      </c>
+      <c r="C64" s="205" t="s">
         <v>194</v>
       </c>
-      <c r="B64" s="204" t="s">
-        <v>195</v>
-      </c>
-      <c r="C64" s="205" t="s">
-        <v>196</v>
-      </c>
       <c r="D64" s="206" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="207" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B65" s="208" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C65" s="209" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="D65" s="210" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="211" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B66" s="212" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C66" s="213" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="D66" s="214" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="215" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="B67" s="216" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C67" s="217" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D67" s="218" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="219" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="B68" s="220" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C68" s="221" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D68" s="222" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="223" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B69" s="224" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C69" s="225" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D69" s="226" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="227" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B70" s="228" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C70" s="229" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="D70" s="230" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>